<commit_message>
Quitar curso OS3G y ( no bnilingue)
</commit_message>
<xml_diff>
--- a/Documentación/Estudios_Grupos_Final.xlsx
+++ b/Documentación/Estudios_Grupos_Final.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MSI-PC\Herd\entrada-salida-aseo\Documentación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1E2BAEB-141A-45B8-9AAF-A90983E217FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D12CFCF-016E-43EC-9A36-7956CCEF437D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="86">
   <si>
     <t>descrip. ensenanza</t>
   </si>
@@ -121,9 +121,6 @@
     <t>E3F</t>
   </si>
   <si>
-    <t>OS3G</t>
-  </si>
-  <si>
     <t>E4A</t>
   </si>
   <si>
@@ -200,9 +197,6 @@
   </si>
   <si>
     <t>E3FM</t>
-  </si>
-  <si>
-    <t>ES3GM</t>
   </si>
   <si>
     <t>E4AM</t>
@@ -651,14 +645,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C50"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C49"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="42.453125" customWidth="1"/>
-    <col min="2" max="2" width="17.26953125" customWidth="1"/>
+    <col min="1" max="1" width="76" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -669,7 +663,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -680,7 +674,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -691,7 +685,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -702,7 +696,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -713,7 +707,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -724,7 +718,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -735,7 +729,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -746,7 +740,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -757,7 +751,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>7</v>
       </c>
@@ -765,10 +759,10 @@
         <v>20</v>
       </c>
       <c r="C10" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -776,10 +770,10 @@
         <v>21</v>
       </c>
       <c r="C11" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -787,10 +781,10 @@
         <v>22</v>
       </c>
       <c r="C12" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>7</v>
       </c>
@@ -798,10 +792,10 @@
         <v>23</v>
       </c>
       <c r="C13" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>7</v>
       </c>
@@ -809,10 +803,10 @@
         <v>24</v>
       </c>
       <c r="C14" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>7</v>
       </c>
@@ -820,10 +814,10 @@
         <v>25</v>
       </c>
       <c r="C15" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>7</v>
       </c>
@@ -831,10 +825,10 @@
         <v>26</v>
       </c>
       <c r="C16" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>7</v>
       </c>
@@ -842,10 +836,10 @@
         <v>27</v>
       </c>
       <c r="C17" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>7</v>
       </c>
@@ -853,10 +847,10 @@
         <v>28</v>
       </c>
       <c r="C18" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>7</v>
       </c>
@@ -864,10 +858,10 @@
         <v>29</v>
       </c>
       <c r="C19" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>7</v>
       </c>
@@ -875,10 +869,10 @@
         <v>30</v>
       </c>
       <c r="C20" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>7</v>
       </c>
@@ -886,10 +880,10 @@
         <v>31</v>
       </c>
       <c r="C21" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>7</v>
       </c>
@@ -897,10 +891,10 @@
         <v>32</v>
       </c>
       <c r="C22" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>7</v>
       </c>
@@ -908,10 +902,10 @@
         <v>33</v>
       </c>
       <c r="C23" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>7</v>
       </c>
@@ -919,10 +913,10 @@
         <v>34</v>
       </c>
       <c r="C24" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>7</v>
       </c>
@@ -930,10 +924,10 @@
         <v>35</v>
       </c>
       <c r="C25" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>7</v>
       </c>
@@ -941,10 +935,10 @@
         <v>36</v>
       </c>
       <c r="C26" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>7</v>
       </c>
@@ -952,131 +946,131 @@
         <v>37</v>
       </c>
       <c r="C27" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B28" t="s">
         <v>38</v>
       </c>
       <c r="C28" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B29" t="s">
+        <v>20</v>
+      </c>
+      <c r="C29" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>8</v>
-      </c>
-      <c r="B29" t="s">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>8</v>
+      </c>
+      <c r="B30" t="s">
+        <v>21</v>
+      </c>
+      <c r="C30" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>8</v>
+      </c>
+      <c r="B31" t="s">
         <v>39</v>
       </c>
-      <c r="C29" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>8</v>
-      </c>
-      <c r="B30" t="s">
-        <v>20</v>
-      </c>
-      <c r="C30" t="s">
+      <c r="C31" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
-        <v>8</v>
-      </c>
-      <c r="B31" t="s">
-        <v>21</v>
-      </c>
-      <c r="C31" t="s">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>8</v>
+      </c>
+      <c r="B32" t="s">
+        <v>25</v>
+      </c>
+      <c r="C32" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
-        <v>8</v>
-      </c>
-      <c r="B32" t="s">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>8</v>
+      </c>
+      <c r="B33" t="s">
+        <v>26</v>
+      </c>
+      <c r="C33" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>8</v>
+      </c>
+      <c r="B34" t="s">
         <v>40</v>
       </c>
-      <c r="C32" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>8</v>
-      </c>
-      <c r="B33" t="s">
-        <v>25</v>
-      </c>
-      <c r="C33" t="s">
+      <c r="C34" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>8</v>
-      </c>
-      <c r="B34" t="s">
-        <v>26</v>
-      </c>
-      <c r="C34" t="s">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>8</v>
+      </c>
+      <c r="B35" t="s">
+        <v>30</v>
+      </c>
+      <c r="C35" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
-        <v>8</v>
-      </c>
-      <c r="B35" t="s">
-        <v>41</v>
-      </c>
-      <c r="C35" t="s">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>8</v>
+      </c>
+      <c r="B36" t="s">
+        <v>31</v>
+      </c>
+      <c r="C36" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
-        <v>8</v>
-      </c>
-      <c r="B36" t="s">
-        <v>30</v>
-      </c>
-      <c r="C36" t="s">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>8</v>
+      </c>
+      <c r="B37" t="s">
+        <v>32</v>
+      </c>
+      <c r="C37" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
-        <v>8</v>
-      </c>
-      <c r="B37" t="s">
-        <v>31</v>
-      </c>
-      <c r="C37" t="s">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>8</v>
+      </c>
+      <c r="B38" t="s">
+        <v>33</v>
+      </c>
+      <c r="C38" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
-        <v>8</v>
-      </c>
-      <c r="B38" t="s">
-        <v>32</v>
-      </c>
-      <c r="C38" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>8</v>
       </c>
@@ -1084,10 +1078,10 @@
         <v>34</v>
       </c>
       <c r="C39" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>8</v>
       </c>
@@ -1095,10 +1089,10 @@
         <v>35</v>
       </c>
       <c r="C40" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>8</v>
       </c>
@@ -1106,21 +1100,21 @@
         <v>36</v>
       </c>
       <c r="C41" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>9</v>
+      </c>
+      <c r="B42" t="s">
+        <v>41</v>
+      </c>
+      <c r="C42" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
-        <v>8</v>
-      </c>
-      <c r="B42" t="s">
-        <v>37</v>
-      </c>
-      <c r="C42" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>9</v>
       </c>
@@ -1128,10 +1122,10 @@
         <v>42</v>
       </c>
       <c r="C43" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>9</v>
       </c>
@@ -1139,73 +1133,62 @@
         <v>43</v>
       </c>
       <c r="C44" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>10</v>
+      </c>
+      <c r="B45" t="s">
+        <v>41</v>
+      </c>
+      <c r="C45" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
-        <v>9</v>
-      </c>
-      <c r="B45" t="s">
-        <v>44</v>
-      </c>
-      <c r="C45" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>10</v>
       </c>
       <c r="B46" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C46" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B47" t="s">
         <v>45</v>
       </c>
       <c r="C47" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>11</v>
       </c>
       <c r="B48" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C48" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B49" t="s">
         <v>43</v>
       </c>
       <c r="C49" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
-        <v>10</v>
-      </c>
-      <c r="B50" t="s">
-        <v>44</v>
-      </c>
-      <c r="C50" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Vista de nombre del curso completo en excepciones medicas, alumnos
</commit_message>
<xml_diff>
--- a/Documentación/Estudios_Grupos_Final.xlsx
+++ b/Documentación/Estudios_Grupos_Final.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MSI-PC\Herd\entrada-salida-aseo\Documentación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D12CFCF-016E-43EC-9A36-7956CCEF437D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9917F1E-8010-4C59-8092-87FEAA73DBC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5235" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -284,7 +284,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -294,6 +294,14 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -336,11 +344,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -645,7 +654,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="76" customWidth="1"/>
@@ -665,90 +674,90 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>16</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>17</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C9" t="s">
-        <v>19</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -756,10 +765,10 @@
         <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C10" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -767,10 +776,10 @@
         <v>7</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C11" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -778,43 +787,43 @@
         <v>7</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="C12" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B13" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="C13" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B14" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C14" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B15" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C15" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -822,373 +831,375 @@
         <v>7</v>
       </c>
       <c r="B16" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C16" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>7</v>
       </c>
       <c r="B17" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C17" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>7</v>
       </c>
       <c r="B18" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C18" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>7</v>
       </c>
       <c r="B19" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C19" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>7</v>
       </c>
       <c r="B20" t="s">
+        <v>32</v>
+      </c>
+      <c r="C20" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>8</v>
+      </c>
+      <c r="B21" t="s">
+        <v>40</v>
+      </c>
+      <c r="C21" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>8</v>
+      </c>
+      <c r="B22" t="s">
         <v>30</v>
       </c>
-      <c r="C20" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>7</v>
-      </c>
-      <c r="B21" t="s">
+      <c r="C22" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>8</v>
+      </c>
+      <c r="B23" t="s">
         <v>31</v>
       </c>
-      <c r="C21" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>7</v>
-      </c>
-      <c r="B22" t="s">
+      <c r="C23" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B24" t="s">
         <v>32</v>
       </c>
-      <c r="C22" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>7</v>
-      </c>
-      <c r="B23" t="s">
+      <c r="C24" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" t="s">
         <v>33</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C25" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>7</v>
-      </c>
-      <c r="B24" t="s">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" t="s">
         <v>34</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C26" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>7</v>
-      </c>
-      <c r="B25" t="s">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>7</v>
+      </c>
+      <c r="B27" t="s">
         <v>35</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C27" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>7</v>
-      </c>
-      <c r="B26" t="s">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>7</v>
+      </c>
+      <c r="B28" t="s">
         <v>36</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C28" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>7</v>
-      </c>
-      <c r="B27" t="s">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>7</v>
+      </c>
+      <c r="B29" t="s">
         <v>37</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C29" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>8</v>
-      </c>
-      <c r="B28" t="s">
-        <v>38</v>
-      </c>
-      <c r="C28" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>8</v>
-      </c>
-      <c r="B29" t="s">
-        <v>20</v>
-      </c>
-      <c r="C29" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="F29" s="2"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>8</v>
       </c>
       <c r="B30" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="C30" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>8</v>
       </c>
       <c r="B31" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C31" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>8</v>
       </c>
       <c r="B32" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="C32" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>8</v>
       </c>
       <c r="B33" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="C33" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B34" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C34" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B35" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="C35" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B36" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="C36" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B37" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="C37" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B38" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="C38" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B39" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="C39" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B40" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="C40" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B41" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C41" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="B42" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="C42" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="I42" s="2"/>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="B43" t="s">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="C43" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="B44" t="s">
-        <v>43</v>
+        <v>13</v>
       </c>
       <c r="C44" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="B45" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="C45" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B46" t="s">
-        <v>44</v>
+        <v>16</v>
       </c>
       <c r="C46" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B47" t="s">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="C47" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B48" t="s">
-        <v>42</v>
+        <v>18</v>
       </c>
       <c r="C48" t="s">
-        <v>84</v>
+        <v>18</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B49" t="s">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="C49" t="s">
-        <v>85</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
campo nombreUsuario, nuevos usuarios y bienvenida en el dashboard
</commit_message>
<xml_diff>
--- a/Documentación/Estudios_Grupos_Final.xlsx
+++ b/Documentación/Estudios_Grupos_Final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MSI-PC\Herd\entrada-salida-aseo\Documentación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9917F1E-8010-4C59-8092-87FEAA73DBC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1641924-3108-4788-8FB3-5E3FA6082D18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,18 +31,6 @@
     <t>subgrupo</t>
   </si>
   <si>
-    <t>Informática y comunicaciones</t>
-  </si>
-  <si>
-    <t>Mantenimiento de vehículos</t>
-  </si>
-  <si>
-    <t>Sistemas Microinformáticos y Redes</t>
-  </si>
-  <si>
-    <t>Desarrollo de Aplicaciones Web</t>
-  </si>
-  <si>
     <t>Educación Secundaria Obligatoria  Programa de Mejora en Lenguas Extranjeras</t>
   </si>
   <si>
@@ -278,6 +266,18 @@
   </si>
   <si>
     <t>B2BHS</t>
+  </si>
+  <si>
+    <t>Informática y comunicaciones (IC)</t>
+  </si>
+  <si>
+    <t>Mantenimiento de vehículos (MV)</t>
+  </si>
+  <si>
+    <t>Sistemas Microinformáticos y Redes (SMR)</t>
+  </si>
+  <si>
+    <t>Desarrollo de Aplicaciones Web (DAW)</t>
   </si>
 </sst>
 </file>
@@ -674,532 +674,532 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C7" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C9" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C10" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C11" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C12" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B13" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C13" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C14" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C15" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B16" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C16" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B17" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C17" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C18" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B19" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C19" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B20" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C20" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B21" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C21" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B22" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C22" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B23" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C23" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B24" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C24" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B25" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C25" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B26" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C26" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B27" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C27" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B28" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C28" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="B29" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C29" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F29" s="2"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B30" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C30" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B31" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C31" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B32" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C32" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B33" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="C33" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B34" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C34" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B35" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C35" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B36" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C36" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B37" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C37" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B38" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C38" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B39" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C39" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B40" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C40" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B41" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C41" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>3</v>
+        <v>82</v>
       </c>
       <c r="B42" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C42" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="I42" s="2"/>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>3</v>
+        <v>82</v>
       </c>
       <c r="B43" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C43" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>4</v>
+        <v>83</v>
       </c>
       <c r="B44" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C44" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>4</v>
+        <v>83</v>
       </c>
       <c r="B45" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C45" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>5</v>
+        <v>84</v>
       </c>
       <c r="B46" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C46" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>5</v>
+        <v>84</v>
       </c>
       <c r="B47" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C47" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>6</v>
+        <v>85</v>
       </c>
       <c r="B48" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C48" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>6</v>
-      </c>
-      <c r="B49" t="s">
-        <v>19</v>
+        <v>85</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="C49" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>